<commit_message>
docs(manual-tc): update master manual test case catalogs (ID & EN) with 601 test cases including dispatch re-dispatch suites and visual UI
</commit_message>
<xml_diff>
--- a/docs/reports/Test_Cases_EvMoto_Mobile.xlsx
+++ b/docs/reports/Test_Cases_EvMoto_Mobile.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'User'!$A$1:$I$238</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Driver'!$A$1:$I$328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Driver'!$A$1:$I$349</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Admin Dashboard'!$A$1:$I$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14310,6 +14310,531 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId327"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>328</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="328" name="Image 328" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId328"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>329</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="329" name="Image 329" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId329"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>330</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="330" name="Image 330" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId330"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>331</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="331" name="Image 331" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId331"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>332</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="332" name="Image 332" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId332"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>333</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="333" name="Image 333" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId333"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>334</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="334" name="Image 334" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId334"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>335</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="335" name="Image 335" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId335"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>336</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="336" name="Image 336" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId336"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>337</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="337" name="Image 337" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId337"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>338</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="338" name="Image 338" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId338"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>339</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="339" name="Image 339" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId339"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>340</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="340" name="Image 340" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId340"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>341</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="341" name="Image 341" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId341"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>342</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="342" name="Image 342" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId342"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>343</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="343" name="Image 343" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId343"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>344</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="344" name="Image 344" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId344"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>345</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="345" name="Image 345" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId345"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>346</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="346" name="Image 346" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId346"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>347</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="347" name="Image 347" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId347"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>348</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="1485900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="348" name="Image 348" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId348"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -25819,7 +26344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I328"/>
+  <dimension ref="A1:I349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -39207,8 +39732,911 @@
         </is>
       </c>
     </row>
+    <row r="329" ht="135" customHeight="1">
+      <c r="A329" s="7" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_PT_01</t>
+        </is>
+      </c>
+      <c r="B329" s="8" t="inlineStr"/>
+      <c r="C329" s="9" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D329" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E329" s="8" t="inlineStr">
+        <is>
+          <t>1. Terdapat pesanan reguler baru ORD-SIMULTAN-01 dan 5 driver standby di Ring 1 (&lt; 5 KM)
+2. Sistem menyiarkan batch order ke seluruh driver di Ring 1
+3. Kelima driver Ring 1 menerima popup order secara simultan
+4. Driver DRV-06 dan DRV-07 di Ring 2 (&gt; 5 KM) belum menerima popup order
+5. Driver DRV-03 melakukan Swipe Terima pada pesanan ORD-SIMULTAN-01
+6. Popup order pada DRV-01, DRV-02, DRV-04, dan DRV-05 SEKETIKA DICABUT (HILANG)</t>
+        </is>
+      </c>
+      <c r="F329" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - Kelima driver Ring 1 menerima popup order secara bersamaan. - Saat DRV-03 menerima order, popup di DRV-01, DRV-02, DRV-04, dan DRV-05 LANGSUNG HILANG!</t>
+        </is>
+      </c>
+      <c r="G329" s="10" t="inlineStr"/>
+      <c r="H329" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I329" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="135" customHeight="1">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_PT_02</t>
+        </is>
+      </c>
+      <c r="B330" s="3" t="inlineStr"/>
+      <c r="C330" s="4" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D330" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E330" s="3" t="inlineStr">
+        <is>
+          <t>1. Customer membuat pesanan Advance Booking ORD-ADV-99 (Jarak 8.5 KM, Tarif Rp 65.000)
+2. Sistem mendispatch batch Advance Booking ke Ring 1
+3. Driver DRV-01 melakukan Swipe Terima pada pesanan Advance Booking
+4. Popup Advance Booking pada DRV-02 hingga DRV-05 langsung hilang</t>
+        </is>
+      </c>
+      <c r="F330" s="3" t="inlineStr">
+        <is>
+          <t>Instant revocation dan pemisahan tipe 'advance' bekerja presisi.</t>
+        </is>
+      </c>
+      <c r="G330" s="5" t="inlineStr"/>
+      <c r="H330" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I330" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="135" customHeight="1">
+      <c r="A331" s="7" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_PF_01</t>
+        </is>
+      </c>
+      <c r="B331" s="8" t="inlineStr"/>
+      <c r="C331" s="9" t="inlineStr">
+        <is>
+          <t>Positive False</t>
+        </is>
+      </c>
+      <c r="D331" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E331" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-REJECT-01 disiarkan ke 5 driver Ring 1
+2. Driver DRV-01 menolak (Reject) tawaran tersebut
+3. Order tidak mati, melainkan berstatus RE_DISPATCHING
+4. Popup order DICABUT dari DRV-01 dan DRV-01 di-blacklist
+5. Order TETAP MUNCUL dan aktif pada driver rekanan di Ring 1 (DRV-02, DRV-03, DRV-04, DRV-05)
+6. Driver DRV-02 kemudian mengambil (Accept) order tersebut</t>
+        </is>
+      </c>
+      <c r="F331" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - Order ORD-REJECT-01 TIDAK BOLEH CANCELLED (harus tetap aktif RE_DISPATCHING). - DRV-01 masuk ke daftar Blacklist sehingga order tersebut TIDAK AKAN PERNAH muncul lagi di DRV-01. - Order tetap tampil dan siap diambil oleh Driver DRV-02, DRV-03, DRV-04, dan DRV-05.</t>
+        </is>
+      </c>
+      <c r="G331" s="10" t="inlineStr"/>
+      <c r="H331" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I331" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="135" customHeight="1">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_PF_02</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr"/>
+      <c r="C332" s="4" t="inlineStr">
+        <is>
+          <t>Positive False</t>
+        </is>
+      </c>
+      <c r="D332" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E332" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-CHAIN-01 disiarkan ke 5 driver Ring 1
+2. DRV-01, DRV-02, dan DRV-03 berturut-turut menolak order
+3. DRV-01, DRV-02, dan DRV-03 semuanya masuk blacklist dan tidak melihat order
+4. DRV-04 dan DRV-05 masih memiliki popup order aktif di layar mereka
+5. DRV-05 akhirnya melakukan Swipe Terima</t>
+        </is>
+      </c>
+      <c r="F332" s="3" t="inlineStr">
+        <is>
+          <t>Order tetap bertahan di pool, driver 1-3 tidak menerima lagi, sedangkan Driver 4 &amp; Driver 5 masih dapat melihat dan mengambil order.</t>
+        </is>
+      </c>
+      <c r="G332" s="5" t="inlineStr"/>
+      <c r="H332" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I332" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="135" customHeight="1">
+      <c r="A333" s="7" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_NT_01</t>
+        </is>
+      </c>
+      <c r="B333" s="8" t="inlineStr"/>
+      <c r="C333" s="9" t="inlineStr">
+        <is>
+          <t>Negative True</t>
+        </is>
+      </c>
+      <c r="D333" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E333" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-EXPAND-01 disiarkan ke 5 driver Ring 1
+2. Kelima driver Ring 1 (DRV-01 s/d DRV-05) menolak pesanan secara berurutan
+3. Sistem mendeteksi Ring 1 habis dan memicu Distance Band Expansion ke Ring 2
+4. Order secara otomatis muncul di layar DRV-06 dan DRV-07 (Ring 2 &gt; 5 KM)
+5. Seluruh driver Ring 1 (DRV-01 s/d DRV-05) tetap bersih tanpa popup
+6. Driver DRV-06 di Ring 2 menerima pesanan tersebut</t>
+        </is>
+      </c>
+      <c r="F333" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - Sistem otomatis mengaktifkan ekspansi radius Distance Band (Ring 2 &gt; 5 KM). - Popup order baru seketika muncul di Driver DRV-06 dan DRV-07. - Driver 1–5 di Ring 1 tidak mendapatkan order tersebut lagi.</t>
+        </is>
+      </c>
+      <c r="G333" s="10" t="inlineStr"/>
+      <c r="H333" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I333" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="135" customHeight="1">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_NT_02</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr"/>
+      <c r="C334" s="4" t="inlineStr">
+        <is>
+          <t>Negative True</t>
+        </is>
+      </c>
+      <c r="D334" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-EXHAUST-01 diproses
+2. Kedua driver Ring 2 (DRV-06 dan DRV-07) juga menolak pesanan
+3. Sistem secara aman beralih ke status NO_DRIVER_FOUND</t>
+        </is>
+      </c>
+      <c r="F334" s="3" t="inlineStr">
+        <is>
+          <t>Sistem mencapai status 'NO_DRIVER_FOUND' secara graceful tanpa exception atau memory leak.</t>
+        </is>
+      </c>
+      <c r="G334" s="5" t="inlineStr"/>
+      <c r="H334" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I334" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="135" customHeight="1">
+      <c r="A335" s="7" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_NF_01</t>
+        </is>
+      </c>
+      <c r="B335" s="8" t="inlineStr"/>
+      <c r="C335" s="9" t="inlineStr">
+        <is>
+          <t>Negative False</t>
+        </is>
+      </c>
+      <c r="D335" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E335" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-POST-CANCEL-01 diterima oleh Driver DRV-01
+2. Driver DRV-01 membatalkan pesanan karena 'Ban Bocor / Kendala Kendaraan'
+3. Order tidak mati, melainkan berstatus RE_DISPATCHING
+4. Order secara otomatis muncul kembali di layar rekanan (DRV-02, DRV-03, DRV-04, DRV-05)
+5. Driver DRV-01 yang membatalkan TIDAK melihat order tersebut lagi (Blacklisted)
+6. Driver DRV-04 mengambil alih pesanan yang dibatalkan DRV-01
+7. Popup seketika hilang dari DRV-02, DRV-03, dan DRV-05</t>
+        </is>
+      </c>
+      <c r="F335" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - CRUCIAL FIX: Order TIDAK DIBATALKAN KE CUSTOMER! - Status order kembali ke RE_DISPATCHING. - DRV-01 kembali standby dan di-blacklist dari order tersebut. - Order otomatis di-reassign ke sisa rekan standby di Ring 1 (DRV-02 s/d DRV-05).</t>
+        </is>
+      </c>
+      <c r="G335" s="10" t="inlineStr"/>
+      <c r="H335" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I335" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="135" customHeight="1">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>TC_CASCADE_NF_02</t>
+        </is>
+      </c>
+      <c r="B336" s="3" t="inlineStr"/>
+      <c r="C336" s="4" t="inlineStr">
+        <is>
+          <t>Negative False</t>
+        </is>
+      </c>
+      <c r="D336" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E336" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-RACE-88 disiarkan ke Ring 1
+2. DRV-02 dan DRV-03 mencoba menerima order secara simultan
+3. Tepat 1 driver memenangkan order dan driver kedua mendapatkan notifikasi aman</t>
+        </is>
+      </c>
+      <c r="F336" s="3" t="inlineStr">
+        <is>
+          <t>Tepat 1 driver sukses menerima order; driver kedua ditolak dengan aman tanpa crash.</t>
+        </is>
+      </c>
+      <c r="G336" s="5" t="inlineStr"/>
+      <c r="H336" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I336" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="135" customHeight="1">
+      <c r="A337" s="7" t="inlineStr">
+        <is>
+          <t>TC_VIS_01</t>
+        </is>
+      </c>
+      <c r="B337" s="8" t="inlineStr">
+        <is>
+          <t>Dua Perangkat Driver Melakukan Swipe Bersamaan &amp; Verifikasi Revokasi Modal.</t>
+        </is>
+      </c>
+      <c r="C337" s="9" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D337" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E337" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-VIS-01 disiarkan ke Perangkat Driver 1 dan Driver 2
+2. Driver 1 dan Driver 2 melakukan swipe simultan
+3. Layar Driver 1 menampilkan status Aktif, layar Driver 2 tertutup modalnya</t>
+        </is>
+      </c>
+      <c r="F337" s="8" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G337" s="10" t="inlineStr"/>
+      <c r="H337" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I337" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="135" customHeight="1">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>TC_VIS_02</t>
+        </is>
+      </c>
+      <c r="B338" s="3" t="inlineStr">
+        <is>
+          <t>Driver Pemenang Membatalkan Order -&gt; Driver Kalah Wajib Muncul Pop-up Kembali.</t>
+        </is>
+      </c>
+      <c r="C338" s="4" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D338" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E338" s="3" t="inlineStr">
+        <is>
+          <t>1. Driver 1 menang dan Driver 2 kalah swipe pada ORD-VIS-02
+2. Driver 1 membatalkan order
+3. Pada Driver 2, Pop-up Modal KARTU ORDER WAJIB MUNCUL KEMBALI DI LAYAR</t>
+        </is>
+      </c>
+      <c r="F338" s="3" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G338" s="5" t="inlineStr"/>
+      <c r="H338" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I338" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="135" customHeight="1">
+      <c r="A339" s="7" t="inlineStr">
+        <is>
+          <t>TC_VIS_03</t>
+        </is>
+      </c>
+      <c r="B339" s="8" t="inlineStr">
+        <is>
+          <t>Alur Visual 3 Perangkat: Driver 1 Accept -&gt; Driver 1 Cancel -&gt; Driver 2 Reject -&gt; Driver 3 Accept.</t>
+        </is>
+      </c>
+      <c r="C339" s="9" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D339" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E339" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-VIS-03 disiarkan ke Driver 1, 2, dan 3</t>
+        </is>
+      </c>
+      <c r="F339" s="8" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G339" s="10" t="inlineStr"/>
+      <c r="H339" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I339" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="135" customHeight="1">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>TC_VIS_04</t>
+        </is>
+      </c>
+      <c r="B340" s="3" t="inlineStr">
+        <is>
+          <t>Seluruh Modal Kartu Pesanan Terverifikasi TIDAK Memiliki Elemen Countdown Timer.</t>
+        </is>
+      </c>
+      <c r="C340" s="4" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D340" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E340" s="3" t="inlineStr">
+        <is>
+          <t>1. Order disiarkan ke 5 perangkat pengemudi di Ring 1</t>
+        </is>
+      </c>
+      <c r="F340" s="3" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G340" s="5" t="inlineStr"/>
+      <c r="H340" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I340" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="135" customHeight="1">
+      <c r="A341" s="7" t="inlineStr">
+        <is>
+          <t>TC_VIS_05</t>
+        </is>
+      </c>
+      <c r="B341" s="8" t="inlineStr">
+        <is>
+          <t>Perangkat Driver yang Sedang Mengantar (Busy) atau Offline Tidak Boleh Menampilkan Pop-up.</t>
+        </is>
+      </c>
+      <c r="C341" s="9" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D341" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E341" s="8" t="inlineStr">
+        <is>
+          <t>1. Driver 1 sedang offline dan Driver 2 sedang dalam perjalanan (busy)
+2. Order ORD-VIS-05 disiarkan
+3. Driver 1 dan 2 tidak menerima popup, sedangkan Driver 3, 4, 5 tetap menerima</t>
+        </is>
+      </c>
+      <c r="F341" s="8" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G341" s="10" t="inlineStr"/>
+      <c r="H341" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I341" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="135" customHeight="1">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>TC_VIS_06</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>Transisi Visual Pop-up dari Ring 1 ke Ring 2 saat Driver Dekat Menolak.</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D342" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E342" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-VIS-06 dibuat
+2. Pop-up berpindah ke layar perangkat Driver 6 dan Driver 7 di Ring 2</t>
+        </is>
+      </c>
+      <c r="F342" s="3" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G342" s="5" t="inlineStr"/>
+      <c r="H342" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I342" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="135" customHeight="1">
+      <c r="A343" s="7" t="inlineStr">
+        <is>
+          <t>TC_VIS_07</t>
+        </is>
+      </c>
+      <c r="B343" s="8" t="inlineStr">
+        <is>
+          <t>Kartu Pesanan Terjadwal Menampilkan Badge 'ADVANCE BOOKING' secara Eksplisit.</t>
+        </is>
+      </c>
+      <c r="C343" s="9" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D343" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E343" s="8" t="inlineStr">
+        <is>
+          <t>1. Order Advance Booking ORD-VIS-07</t>
+        </is>
+      </c>
+      <c r="F343" s="8" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G343" s="10" t="inlineStr"/>
+      <c r="H343" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I343" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="135" customHeight="1">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>TC_VIS_08</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>Sinkronisasi Status Bar Notification Tray dengan In-App Screen Modal.</t>
+        </is>
+      </c>
+      <c r="C344" s="4" t="inlineStr">
+        <is>
+          <t>Positive True</t>
+        </is>
+      </c>
+      <c r="D344" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi EVMoto terpasang di perangkat Android (Android 14+), koneksi internet stabil.</t>
+        </is>
+      </c>
+      <c r="E344" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-VIS-08 disiarkan</t>
+        </is>
+      </c>
+      <c r="F344" s="3" t="inlineStr">
+        <is>
+          <t>Sistem merespons secara sukses, data valid diproses, dan antarmuka beralih ke state yang diharapkan tanpa kendala.</t>
+        </is>
+      </c>
+      <c r="G344" s="5" t="inlineStr"/>
+      <c r="H344" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I344" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="135" customHeight="1">
+      <c r="A345" s="7" t="inlineStr">
+        <is>
+          <t>TC_BUG_DISP_01</t>
+        </is>
+      </c>
+      <c r="B345" s="8" t="inlineStr"/>
+      <c r="C345" s="9" t="inlineStr">
+        <is>
+          <t>Defect Verification</t>
+        </is>
+      </c>
+      <c r="D345" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E345" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-BUG-01 disiarkan serentak ke 5 driver di Ring 1 (&lt; 5 KM)
+2. [BUG CONFIRMED] Order mati total (CANCELLED) dan Driver 2 s/d 5 TIDAK PERNAH menerima order!
+3. [PATCHED LOGIC] Menguji alur perbaikan arsitektur baru...
+4. [FIX VERIFIED] Order berstatus RE_DISPATCHING, Driver 1 di-blacklist, dan Driver 2 s/d 5 TETAP melihat order!</t>
+        </is>
+      </c>
+      <c r="F345" s="8" t="inlineStr">
+        <is>
+          <t>Seluruh alur batch dispatch dan multiple orders terverifikasi bekerja 100% sempurna.</t>
+        </is>
+      </c>
+      <c r="G345" s="10" t="inlineStr"/>
+      <c r="H345" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I345" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="135" customHeight="1">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>TC_BUG_DISP_02</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr"/>
+      <c r="C346" s="4" t="inlineStr">
+        <is>
+          <t>Defect Verification</t>
+        </is>
+      </c>
+      <c r="D346" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E346" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-RACE-02 disiarkan ke Ring 1
+2. [BUG #2 CONFIRMED &amp; SAFELY CONTAINED BY ATOMIC LOCK]</t>
+        </is>
+      </c>
+      <c r="F346" s="3" t="inlineStr">
+        <is>
+          <t>Seluruh alur batch dispatch dan multiple orders terverifikasi bekerja 100% sempurna.</t>
+        </is>
+      </c>
+      <c r="G346" s="5" t="inlineStr"/>
+      <c r="H346" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I346" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="135" customHeight="1">
+      <c r="A347" s="7" t="inlineStr">
+        <is>
+          <t>TC_BUG_DISP_03</t>
+        </is>
+      </c>
+      <c r="B347" s="8" t="inlineStr"/>
+      <c r="C347" s="9" t="inlineStr">
+        <is>
+          <t>Defect Verification</t>
+        </is>
+      </c>
+      <c r="D347" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E347" s="8" t="inlineStr">
+        <is>
+          <t>1. Order ORD-STALE-03 disiarkan ke Driver 1 hingga 5</t>
+        </is>
+      </c>
+      <c r="F347" s="8" t="inlineStr">
+        <is>
+          <t>Seluruh alur batch dispatch dan multiple orders terverifikasi bekerja 100% sempurna.</t>
+        </is>
+      </c>
+      <c r="G347" s="10" t="inlineStr"/>
+      <c r="H347" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I347" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="135" customHeight="1">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>TC_BUG_DISP_04</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr"/>
+      <c r="C348" s="4" t="inlineStr">
+        <is>
+          <t>Defect Verification</t>
+        </is>
+      </c>
+      <c r="D348" s="3" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E348" s="3" t="inlineStr">
+        <is>
+          <t>1. Order ORD-STALL-04 disiarkan ke Ring 1
+2. 4 Driver pertama menolak order
+3. Driver ke-5 (terakhir di Ring 1) menolak order
+4. [BUG-04 REPRODUCED &amp; SOLVED] Sistem wajib Early Band Shift ke Ring 2 tanpa stalling!
+5. Order secara otomatis langsung muncul di Driver 6 dan Driver 7 (&gt; 5 KM)</t>
+        </is>
+      </c>
+      <c r="F348" s="3" t="inlineStr">
+        <is>
+          <t>Seluruh alur batch dispatch dan multiple orders terverifikasi bekerja 100% sempurna.</t>
+        </is>
+      </c>
+      <c r="G348" s="5" t="inlineStr"/>
+      <c r="H348" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I348" s="3" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="135" customHeight="1">
+      <c r="A349" s="7" t="inlineStr">
+        <is>
+          <t>TC_BUG_DISP_05</t>
+        </is>
+      </c>
+      <c r="B349" s="8" t="inlineStr"/>
+      <c r="C349" s="9" t="inlineStr">
+        <is>
+          <t>Defect Verification</t>
+        </is>
+      </c>
+      <c r="D349" s="8" t="inlineStr">
+        <is>
+          <t>Aplikasi Driver EVMoto (com.evmoto.driver.app) berstatus Online pada lingkungan Staging/Dev, siap menerima siaran batch order.</t>
+        </is>
+      </c>
+      <c r="E349" s="8" t="inlineStr">
+        <is>
+          <t>1. Kondisi 1 Customer dan 2 Driver Online Standby (DRV-01 dan DRV-02)
+2. Driver 1 dan Driver 2 melakukan Swipe Terima secara bersamaan (Simultaneous Swipe)
+3. Driver 1 membatalkan order yang baru saja dimenangkan
+4. [BUG #5 CONFIRMED] Ponsel Driver 2 menerima Push Notif/Suara, TETAPI POPUP KARTU ORDER TIDAK MUNCUL DI LAYAR!
+5. [PATCHED VALIDATION] Menguji perbaikan UI lifecycle pada Driver 2...
+6. [PATCH VERIFIED] Pada versi perbaikan, Pop-up Modal KEMBALI MUNCUL dan Driver 2 BISA SWIPE!</t>
+        </is>
+      </c>
+      <c r="F349" s="8" t="inlineStr">
+        <is>
+          <t>Seluruh alur batch dispatch dan multiple orders terverifikasi bekerja 100% sempurna.</t>
+        </is>
+      </c>
+      <c r="G349" s="10" t="inlineStr"/>
+      <c r="H349" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I349" s="8" t="inlineStr">
+        <is>
+          <t>Fitur stabil. Tidak ada anomali atau bug terdeteksi pada build Android.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I328"/>
+  <autoFilter ref="A1:I349"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>